<commit_message>
Update data.xlsx with new contact info
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kiuchi-my.sharepoint.com/personal/isozaki_kiuchi_co_jp/Documents/fmsf-phone/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kiuchi-my.sharepoint.com/personal/isozaki_kiuchi_co_jp/Documents/FMSF-Direct-line/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="843" documentId="8_{F85A9A68-4E93-4088-9ED5-1903CFFF7F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{857474ED-1FD6-4EB1-814C-A8E22AC0EE30}"/>
+  <xr:revisionPtr revIDLastSave="848" documentId="8_{F85A9A68-4E93-4088-9ED5-1903CFFF7F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9311776B-EB00-47F4-9764-E61527219151}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D411879D-5147-439A-8907-627E102D99C2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1576" uniqueCount="1054">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1581" uniqueCount="1058">
   <si>
     <t>氏名</t>
   </si>
@@ -4248,6 +4248,34 @@
   </si>
   <si>
     <t>awata@ys-h.co.jp</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>現場事務員</t>
+    <rPh sb="0" eb="5">
+      <t>ゲンバジムイン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>事務</t>
+    <rPh sb="0" eb="2">
+      <t>ジム</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>磯﨑 艶子</t>
+    <rPh sb="0" eb="2">
+      <t>イソザキ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ツヤコ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>080-2605-5075</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -4359,10 +4387,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4682,7 +4706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CED22340-6398-430F-AD0F-E88DFD8C2F52}">
-  <dimension ref="A1:J184"/>
+  <dimension ref="A1:J185"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="2" width="8.9140625" customWidth="1"/>
@@ -9795,6 +9819,23 @@
       </c>
       <c r="I184" t="s">
         <v>1047</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A185" t="s">
+        <v>1054</v>
+      </c>
+      <c r="C185" t="s">
+        <v>913</v>
+      </c>
+      <c r="D185" t="s">
+        <v>1055</v>
+      </c>
+      <c r="E185" t="s">
+        <v>1056</v>
+      </c>
+      <c r="I185" t="s">
+        <v>1057</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data.xlsx to trigger workflow
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kiuchi-my.sharepoint.com/personal/isozaki_kiuchi_co_jp/Documents/FMSF-Direct-line/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="848" documentId="8_{F85A9A68-4E93-4088-9ED5-1903CFFF7F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9311776B-EB00-47F4-9764-E61527219151}"/>
+  <xr:revisionPtr revIDLastSave="853" documentId="8_{F85A9A68-4E93-4088-9ED5-1903CFFF7F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6989B90-6A57-4B70-8A28-D34CAAA6E246}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D411879D-5147-439A-8907-627E102D99C2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1581" uniqueCount="1058">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1576" uniqueCount="1054">
   <si>
     <t>氏名</t>
   </si>
@@ -4248,34 +4248,6 @@
   </si>
   <si>
     <t>awata@ys-h.co.jp</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>現場事務員</t>
-    <rPh sb="0" eb="5">
-      <t>ゲンバジムイン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>事務</t>
-    <rPh sb="0" eb="2">
-      <t>ジム</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>磯﨑 艶子</t>
-    <rPh sb="0" eb="2">
-      <t>イソザキ</t>
-    </rPh>
-    <rPh sb="3" eb="5">
-      <t>ツヤコ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>080-2605-5075</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -4387,6 +4359,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4706,11 +4682,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CED22340-6398-430F-AD0F-E88DFD8C2F52}">
-  <dimension ref="A1:J185"/>
+  <dimension ref="A1:J184"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="2" width="8.9140625" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
     <col min="5" max="5" width="15.08203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9819,23 +9795,6 @@
       </c>
       <c r="I184" t="s">
         <v>1047</v>
-      </c>
-    </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A185" t="s">
-        <v>1054</v>
-      </c>
-      <c r="C185" t="s">
-        <v>913</v>
-      </c>
-      <c r="D185" t="s">
-        <v>1055</v>
-      </c>
-      <c r="E185" t="s">
-        <v>1056</v>
-      </c>
-      <c r="I185" t="s">
-        <v>1057</v>
       </c>
     </row>
   </sheetData>

</xml_diff>